<commit_message>
Inspiration Module support, fix Hub Spoke name-sync bugs, rename hubSpokesNM, and drop post-save back-navigation~
</commit_message>
<xml_diff>
--- a/brief-template.xlsx
+++ b/brief-template.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Item Carousel" sheetId="8" r:id="rId8"/>
     <sheet name="YouTube" sheetId="9" r:id="rId9"/>
     <sheet name="Recipe" sheetId="10" r:id="rId10"/>
+    <sheet name="Inspiration Module" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -638,6 +639,739 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AK6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Order</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Need Edit Web</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Title EN</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Title FR</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Card 1 Image EN Image</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Card 1 Image EN Alt</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Card 1 Image FR Image</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Card 1 Image FR Alt</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Card 1 Heading EN</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Card 1 Heading FR</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Card 1 Sub-Heading EN</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Card 1 Sub-Heading FR</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Card 1 Link URL EN</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Card 1 Link URL FR</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Card 1 SKUs (one per line)</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Card 2 Image EN Image</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Card 2 Image EN Alt</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Card 2 Image FR Image</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Card 2 Image FR Alt</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Card 2 Heading EN</v>
+      </c>
+      <c r="U1" t="str">
+        <v>Card 2 Heading FR</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Card 2 Sub-Heading EN</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Card 2 Sub-Heading FR</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Card 2 Link URL EN</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Card 2 Link URL FR</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Card 2 SKUs (one per line)</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Card 3 Image EN Image</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Card 3 Image EN Alt</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>Card 3 Image FR Image</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Card 3 Image FR Alt</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>Card 3 Heading EN</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Card 3 Heading FR</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Card 3 Sub-Heading EN</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>Card 3 Sub-Heading FR</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>Card 3 Link URL EN</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>Card 3 Link URL FR</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>Card 3 SKUs (one per line)</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2">
+        <v>20</v>
+      </c>
+      <c r="B2" t="b">
+        <v>0</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Shop</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Magasiner</v>
+      </c>
+      <c r="E2" t="str">
+        <v>INSPO-1-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_E.jpg</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Febreze Air</v>
+      </c>
+      <c r="G2" t="str">
+        <v>INSPO-1-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_F.jpg</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Febreze Air</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Febreze Air</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Febreze Air</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Just-cleaned freshness in every space.</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Pour une sensation de fraîcheur dans chaque espace.</v>
+      </c>
+      <c r="M2" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="O2" t="str" xml:space="preserve">
+        <v xml:space="preserve">4VV5VAC48801
+6000197848660
+6000197849110
+6000208807431
+6000196727537
+6000196727398
+6000206703073
+7BBC9XXXC8G8
+575R6JXDFP2H
+6000199303948</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
+      </c>
+      <c r="AA2" t="str">
+        <v/>
+      </c>
+      <c r="AB2" t="str">
+        <v/>
+      </c>
+      <c r="AC2" t="str">
+        <v/>
+      </c>
+      <c r="AD2" t="str">
+        <v/>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
+        <v/>
+      </c>
+      <c r="AG2" t="str">
+        <v/>
+      </c>
+      <c r="AH2" t="str">
+        <v/>
+      </c>
+      <c r="AI2" t="str">
+        <v/>
+      </c>
+      <c r="AJ2" t="str">
+        <v/>
+      </c>
+      <c r="AK2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3">
+        <v>21</v>
+      </c>
+      <c r="B3" t="b">
+        <v>0</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Shop</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Magasiner</v>
+      </c>
+      <c r="E3" t="str">
+        <v>INSPO-2-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_E.jpg</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Febreze Plug</v>
+      </c>
+      <c r="G3" t="str">
+        <v>INSPO-2-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_F.jpg</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Prise Febreze</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Febreze Plug</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Prise Febreze</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Up to 50 days of continuous fragrance.</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Jusqu'à 50 jours de parfum continu.</v>
+      </c>
+      <c r="M3" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="N3" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="O3" t="str" xml:space="preserve">
+        <v xml:space="preserve">6000202392680
+0TBOFWY48G5X
+6000208170948
+6000208807841
+6000200692396
+6000208626369
+6000208808680
+6000208808911
+16R9X4DM2FMG
+6000208807734</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+      <c r="X3" t="str">
+        <v/>
+      </c>
+      <c r="Y3" t="str">
+        <v/>
+      </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
+      <c r="AA3" t="str">
+        <v/>
+      </c>
+      <c r="AB3" t="str">
+        <v/>
+      </c>
+      <c r="AC3" t="str">
+        <v/>
+      </c>
+      <c r="AD3" t="str">
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
+        <v/>
+      </c>
+      <c r="AG3" t="str">
+        <v/>
+      </c>
+      <c r="AH3" t="str">
+        <v/>
+      </c>
+      <c r="AI3" t="str">
+        <v/>
+      </c>
+      <c r="AJ3" t="str">
+        <v/>
+      </c>
+      <c r="AK3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4">
+        <v>22</v>
+      </c>
+      <c r="B4" t="b">
+        <v>0</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Shop</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Magasiner</v>
+      </c>
+      <c r="E4" t="str">
+        <v>INSPO-3-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_E.jpg</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Febreze Bathroom</v>
+      </c>
+      <c r="G4" t="str">
+        <v>INSPO-3-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_F.jpg</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Febreze Salle de bain</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Febreze Bathroom</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Febreze Salle de bain</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Non-stop odour-fighting, up to 45 days.</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Élimine les odeurs jusqu'à 45 jours.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="N4" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="O4" t="str" xml:space="preserve">
+        <v xml:space="preserve">6000208807245
+6000208808320
+6000208808307
+6000208807226
+6000208808621
+5GK8XSRLL6B4
+6000208807974
+6000208807906
+6000208806916
+1J23J1EOL8CL</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
+      <c r="AA4" t="str">
+        <v/>
+      </c>
+      <c r="AB4" t="str">
+        <v/>
+      </c>
+      <c r="AC4" t="str">
+        <v/>
+      </c>
+      <c r="AD4" t="str">
+        <v/>
+      </c>
+      <c r="AE4" t="str">
+        <v/>
+      </c>
+      <c r="AF4" t="str">
+        <v/>
+      </c>
+      <c r="AG4" t="str">
+        <v/>
+      </c>
+      <c r="AH4" t="str">
+        <v/>
+      </c>
+      <c r="AI4" t="str">
+        <v/>
+      </c>
+      <c r="AJ4" t="str">
+        <v/>
+      </c>
+      <c r="AK4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5">
+        <v>23</v>
+      </c>
+      <c r="B5" t="b">
+        <v>0</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Shop</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Magasiner</v>
+      </c>
+      <c r="E5" t="str">
+        <v>INSPO-4-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_E.jpg</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Febreze Auto</v>
+      </c>
+      <c r="G5" t="str">
+        <v>INSPO-4-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_F.jpg</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Febreze Auto</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Febreze Auto</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Febreze Auto</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Eliminate odours for better rides.</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Roulez sans odeurs désagréables.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="O5" t="str" xml:space="preserve">
+        <v xml:space="preserve">6000197850023
+6000208807987
+6000199312941
+6000208806981
+6000208806836
+6000199315800
+6000208418483
+6000208808592
+6000208419850
+6000208419543</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
+      </c>
+      <c r="AA5" t="str">
+        <v/>
+      </c>
+      <c r="AB5" t="str">
+        <v/>
+      </c>
+      <c r="AC5" t="str">
+        <v/>
+      </c>
+      <c r="AD5" t="str">
+        <v/>
+      </c>
+      <c r="AE5" t="str">
+        <v/>
+      </c>
+      <c r="AF5" t="str">
+        <v/>
+      </c>
+      <c r="AG5" t="str">
+        <v/>
+      </c>
+      <c r="AH5" t="str">
+        <v/>
+      </c>
+      <c r="AI5" t="str">
+        <v/>
+      </c>
+      <c r="AJ5" t="str">
+        <v/>
+      </c>
+      <c r="AK5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6">
+        <v>24</v>
+      </c>
+      <c r="B6" t="b">
+        <v>0</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Shop</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Magasiner</v>
+      </c>
+      <c r="E6" t="str">
+        <v>INSPO-5-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_E.jpg</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Febreze Fabric</v>
+      </c>
+      <c r="G6" t="str">
+        <v>INSPO-5-BP_CT5231_P&amp;G-Febreze-Brand-Store_261001_F.jpg</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Febreze Tissu</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Febreze Fabric</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Febreze Tissu</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Spray &amp; refresh your household fabrics.</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Vaporisez et rafraîchissez vos tissus d’intérieur.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="N6" t="str">
+        <v>https://www.tbd.com</v>
+      </c>
+      <c r="O6" t="str" xml:space="preserve">
+        <v xml:space="preserve">6000207494286
+6000207362787
+6000208169653
+6000208808480
+6000203371502
+6000207362867
+6000207494519
+6000208808974
+6000207363157</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+      <c r="X6" t="str">
+        <v/>
+      </c>
+      <c r="Y6" t="str">
+        <v/>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
+      </c>
+      <c r="AA6" t="str">
+        <v/>
+      </c>
+      <c r="AB6" t="str">
+        <v/>
+      </c>
+      <c r="AC6" t="str">
+        <v/>
+      </c>
+      <c r="AD6" t="str">
+        <v/>
+      </c>
+      <c r="AE6" t="str">
+        <v/>
+      </c>
+      <c r="AF6" t="str">
+        <v/>
+      </c>
+      <c r="AG6" t="str">
+        <v/>
+      </c>
+      <c r="AH6" t="str">
+        <v/>
+      </c>
+      <c r="AI6" t="str">
+        <v/>
+      </c>
+      <c r="AJ6" t="str">
+        <v/>
+      </c>
+      <c r="AK6" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:AK6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>

</xml_diff>